<commit_message>
Rewrite top-10 reviews and conclusions in plain Russian
Replace telegram-style blurb cells with full stories: what happened,
why, and what it is not. Add a one-piece market intro so 2025 vs 2024
is readable without finance jargon.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_sentyabr_2026.xlsx
+++ b/FMCG_RF_sentyabr_2026.xlsx
@@ -1072,7 +1072,7 @@
   <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -1084,155 +1084,171 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Что происходит на рынке — без телеграфного сжатия</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+          <t>Что происходит на рынке — человеческим языком</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="200" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Если совсем коротко, одной историей. В 2025 году люди в продуктовые магазины ходили и оставляли больше денег, чем в 2024-м. Десятка крупнейших сетей собрала примерно на 16% больше. Это не праздник: цены выросли, сети открывали новые точки, кто-то покупал чужие магазины.
+Но «больше в кассе» не значит «больше в кармане у компании». Кредиты в 2025 году были очень дорогими. Часть того, что покупатель оставил на кассе, ушла банкам в виде процентов. Поэтому у X5 выручка выросла, а прибыль упала. У Магнита выручка тоже выросла, а год закончился убытком. Это не пустые полки и не «сеть разваливается» — это дорогие заёмные деньги.
+Долги у крупных разные. У Ленты долг маленький и даже снизился. У X5 долг есть, но невыбранных кредитов в банках больше, чем сам долг. У Магнита рюкзак тяжёлый: почти полтриллиона чистого долга. Магнит при этом магазины не закрывает и отчётность сдаёт — просто жить так при высокой ставке тяжело.
+С другой стороны прилавка заводы росли медленнее сетей. PepsiCo и Русагро почти сравнялись по продажам. В молочке впервые вышла вперёд «Логика молока» (бывшие заводы Danone). Хард-дискаунтер как формат жив (Чижик у X5 сильно вырос), но сам «Светофор» сжался.
+Все цифры ниже — полный 2025 год к полному 2024-му. 2026-й ещё идёт, годовых отчётов нет, поэтому «на сколько выросли в 2026» в таблице нет.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>П.2. Почему выручка растёт, а прибыль — нет</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Выручка — сколько покупатели оставили в кассе. Прибыль — что осталось компании после зарплат, аренды, закупок и процентов по кредитам. Можно продавать больше и при этом уносить домой меньше: магазины работают, а «цена денег» съедает результат.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="96" customHeight="1">
+    <row r="5" ht="56" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>X5 (Пятёрочка + Перекрёсток + Чижик). Касса выросла на 18,8% до 4,64 трлн ₽ — сеть открывалась и дорожали товары. Чистая прибыль наоборот упала на 13,9% до 94,8 млрд. Компания сама пишет: выросли проценты по долгу (кредиты стали дороже и тело долга больше) и разово отложили 4,1 млрд «на всякий случай», если кто-то из партнёров не расплатится. Плюс X5 щедро вернула деньги акционерам: дивиденды ~159 млрд и выкуп своих акций ~45 млрд. Капитал на балансе сжался, но это не дыра в магазинах, а раздача кэша владельцам. Разбор: vc.ru «Х5 отчиталась за 2025 год. Рост выручки есть, чистая прибыль упала»; пресс-релиз X5 / e-disclosure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="96" customHeight="1">
+          <t>Два разных слова, которые часто путают. Выручка — это сколько покупатели оставили в кассе за год. Прибыль — что осталось компании после зарплат, аренды, закупок товара и, главное, процентов по кредитам. Можно продавать больше и при этом уносить домой меньше: магазины работают, народ покупает, а «цена денег» съедает результат. Именно это и случилось у двух крупнейших сетей.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Магнит. Касса тоже выросла: +15,3% до 3,51 трлн ₽. А вот прибыли нет — чистый убыток 16,6 млрд против прибыли 50 млрд годом раньше. Почему: средневзвешенная ставка по долгу 17,1% (деньги в 2025 были очень дорогими), финансовых расходов 82,3 млрд; минус 3 млрд на курсовых разницах по валютным счетам; плюс покупки «Азбуки вкуса» (29,6 млрд) и «Самбери». Операционное юрлицо АО «Тандер» впервые за 20+ лет ушло в минус (около −22 млрд) — это не «магазины пустые», а проценты по кредитам на развитие. Статьи: «Коммерсантъ» 01.04.2026; РБК про убыток «Тандера».</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
+          <t>X5 — это Пятёрочка, Перекрёсток и Чижик вместе. В кассы за 2025 год пришло 4,64 трлн ₽ — на 18,8% больше, чем в 2024-м. Сеть открывала магазины, товары дорожали, люди не перестали ходить за хлебом и молоком. Казалось бы, отличный год. Но чистая прибыль упала на 13,9% — до 94,8 млрд ₽. Компания сама объясняет почему. Во-первых, кредиты стали дороже, и тело долга больше — банкам ушло больше процентов. Во-вторых, разово отложили 4,1 млрд «на всякий случай», если кто-то из партнёров не расплатится. В-третьих, владельцам щедро вернули деньги: дивиденды около 159 млрд и выкуп своих акций около 45 млрд. Капитал на балансе сжался, но это не дыра в магазинах, а раздача кэша акционерам. Магазины живые. Меньше стало не покупок, а того, что осталось после банков и дивидендов. Где читать: vc.ru «Х5 отчиталась за 2025 год. Рост выручки есть, чистая прибыль упала»; пресс-релиз X5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Коротко: полка живая, народ покупает. Ломается не спрос, а арифметика после процентов. У X5 прибыль ещё плюсовая. У Магнита уже минус. Это разные степени одной болезни — дорогого долга, а не закрытых касс.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+          <t>Магнит. Та же история на кассе и другая внизу отчёта. Выручка +15,3% до 3,51 трлн ₽ — люди покупали. А прибыли нет: убыток 16,6 млрд ₽. Годом раньше была прибыль около 50 млрд. То есть за один год компания перешла из «заработали» в «ушли в минус», хотя магазины не опустели. Почему: деньги в 2025 году стоили очень дорого. Средняя ставка по долгу Магнита — 17,1%, одних только процентов и финансовых расходов набежало 82,3 млрд. Плюс минус 3 млрд на курсе валют. Плюс покупки «Азбуки вкуса» (29,6 млрд) и «Самбери» — это не расходы в кассе магазина, но деньги из группы ушли. Юрлицо, которое реально крутит магазины, — АО «Тандер» — впервые за двадцать с лишним лет закончило год в минусе (около −22 млрд). Это не «покупатели ушли», а проценты по кредитам на развитие. Статьи: «Коммерсантъ» 01.04.2026; РБК про убыток «Тандера».</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Итог этого пункта. Полка живая, народ покупает. Ломается не спрос, а арифметика после процентов по кредитам. У X5 прибыль ещё плюсовая, просто меньше. У Магнита уже минус. Это разные степени одной болезни — дорогого долга, а не закрытых касс.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>П.3. Долги: откуда, перед кем, развалится ли сеть?</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="64" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Что такое «чистый долг» в таблице. Компания должна банкам и/или держателям облигаций (это «весь долг»). На счетах лежит кэш. Чистый долг = весь долг минус кэш. Дальше смотрят, за сколько лет операционная прибыль (EBITDA) этот долг покрыла бы. До 1× — легкий рюкзак. Около 3× — тяжелый, но для ритейла ещё живой. Выше 4–5× без запаса кэша — уже вопрос к выживанию.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="140" customHeight="1">
+    <row r="11" ht="88" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Лента — 48,8 млрд чистого долга. Это не «дыра», а наоборот самый спокойный из крупных. Год назад было 60,9 млрд — долг СНИЗИЛСЯ. Отношение долг/EBITDA 0,6× (меньше года прибыли). Перед кем: на середину 2025 весь долг — банковские кредиты, облигаций у Ленты ещё не было (агентство НКР прямо пишет: «весь долг представлен банковскими кредитами»; компания только собирается выйти на облигации). Имена банков в открытом отчёте пакетом не публикуют — это синдицированные и двусторонние линии крупных российских банков, плюс невыбранный лимит ~226 млрд. На счетах 51,1 млрд кэша — почти столько же, сколько весь короткий долг 55,4 млрд. Рейтинги весны 2026: АКРА AA(RU), НКР и Эксперт РА AA+.ru. Развалится ли? По открытым данным — нет. 48,8 млрд в 23 раза меньше, чем у Магнита; рейтинг «высокая надёжность»; долг падает, а не растёт. Долг появился как у любой крупной сети: товар на складе, стройка магазинов, покупка «Монетки», «Реми», «Улыбки радуги». Это рабочий инструмент, не признак краха. Источники: презентация Ленты 4 кв. 2025; годовой отчёт 2025; пресс-релиз НКР 27.03.2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="128" customHeight="1">
+          <t>Сначала что значит цифра в столбце «чистый долг». Компания должна банкам и/или людям, которые купили её облигации. Это «весь долг». На счетах при этом лежит кэш. Чистый долг = весь долг минус кэш. Если кэша больше, чем долга, в ячейке будет минус — как у Винлаба: это не «минус должна», а запас денег.
+Дальше смотрят простую мерку: за сколько лет обычной операционной прибыли (EBITDA) этот долг можно было бы закрыть. До 1× — лёгкий рюкзак, как небольшая ипотека при нормальной зарплате. Около 3× — уже тяжело, но для большой сети ещё живой. Выше 4–5× без запаса денег на счетах — уже вопрос, потянет ли.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="140" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Магнит — 496 млрд чистого долга (почти ×2 за год). Вот здесь рюкзак тяжёлый. Весь долг 746 млрд: примерно половина — кредиты банков (48,6%), половина — облигации на Московской бирже (50,8%). Перед кем: банки-кредиторы + все, кто купил облигации «Магнита» (фонды, банки, частные инвесторы). Поимённый список держателей бумаг компания не раскрывает — так устроен биржевой рынок. Долг/EBITDA 2,9×. Компания пишет, что во втором полугодии нарочно набрала лишних денег, чтобы заранее закрыть погашения 2026 года (рефинансирование), а не чтобы заткнуть кассовый разрыв. Развалится ли? Признаков дефолта в открытую нет: 33 тысячи магазинов работают, отчётность выходит, облигации торгуются. Но это уже не «комфортный» долг, как у Ленты: если ключевая ставка останется высокой, проценты продолжат съедать прибыль. Следить за 2026 — сможет ли перекредитоваться дешевле. Источники: годовой обзор «Магнита» 2025 (структура долга); «Коммерсантъ» / РБК.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
+          <t>Лента. Чистый долг 48,8 млрд ₽. На фоне Магнита это мелочь, и за год долг даже снизился (было 60,9). Закрыть его хватило бы меньше чем года обычной прибыли. Перед кем должна: только банкам. Облигаций у Ленты в 2025 ещё не было — это прямо пишет рейтинговое агентство НКР. Каким именно банкам — поимённый список в открытый отчёт не кладут, это обычные крупные российские банки плюс невыбранный запас кредитов около 226 млрд. На счетах 51 млрд кэша — почти столько же, сколько короткий долг. Весной 2026 три агентства поставили оценки уровня AA / AA+: «высокая надёжность».
+Развалится ли? По открытым данным — нет. Долг падает, а не растёт; рейтинг хороший; 48,8 млрд в 23 раза меньше, чем у Магнита. Откуда долг вообще взялся: как у любой крупной сети — товар на складе, стройка магазинов, покупка «Монетки», «Реми», «Улыбки радуги». Это рабочий инструмент, не признак краха. Источники: презентация Ленты за 4 кв. 2025, годовой отчёт, пресс-релиз НКР 27.03.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="140" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>X5 — 228,5 млрд чистого долга. Долг/EBITDA 0,84× — лёгкий. Весь долг в рублях. Невыбранные лимиты в крупнейших банках — 773 млрд, на счетах 178 млрд. Перед кем: российские банки и рублёвые облигации (как и у Магнита, без поимённого списка держателей в пресс-релизе). Развалится ли? Нет: запас лимитов больше, чем сам долг. Прибыль упала из-за процентов и дивидендов, а не из-за нехватки покупателей.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="64" customHeight="1">
+          <t>Магнит. Тут рюкзак тяжёлый: чистый долг 496 млрд, почти в два раза больше, чем год назад. Весь долг 746 млрд. Примерно половина — кредиты банков (48,6%), половина — облигации на Московской бирже (50,8%). Перед кем: банки + все, кто купил бумаги «Магнита» (фонды, банки, частные инвесторы). Поимённый список держателей облигаций компания не публикует — так устроен биржевой рынок, бумаги перепродаются.
+Сама компания говорит: во втором полугодии нарочно набрала лишних денег, чтобы заранее закрыть погашения 2026 года, а не потому что в кассах кончились деньги. Признаков дефолта в открытую нет: 33 тысячи магазинов работают, отчётность выходит, облигации торгуются. Но это уже не спокойный долг, как у Ленты. Если ключевая ставка останется высокой, проценты будут и дальше съедать прибыль. За чем следить в 2026-м: сможет ли перекредитоваться дешевле. Источники: годовой обзор Магнита 2025, «Коммерсантъ», РБК.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Mercury (К&amp;Б + Бристоль). Сводного МСФО нет, поэтому чистого долга холдинга в таблице нет — это не «скрыли крах», а не публикуют консолидацию. По юрлицу «Альфа-М» (К&amp;Б) наоборот: с убытка 2024 вышли на прибыль 26 млрд при выручке 847 млрд. Владельцы сняли большие дивиденды — так делают, когда кэш есть, а не когда спасают сеть. В 1 кв. 2026 К&amp;Б впервые чуть сократила число магазинов (−4 точки) — замедление, не развал.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+          <t>X5. Чистый долг 228,5 млрд — заметно меньше Магнита. Рюкзак лёгкий: меньше года прибыли. Весь долг в рублях. Невыбранных кредитов в крупных банках — 773 млрд, то есть запас больше, чем сам долг. На счетах 178 млрд. Перед кем: российские банки и рублёвые облигации, без поимённого списка держателей в пресс-релизе. Развалится ли? Нет. Прибыль упала из-за процентов и дивидендов, а не потому что покупатели ушли.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Mercury — это «Красное &amp; Белое» плюс «Бристоль». Сводного отчёта на весь холдинг нет, поэтому чистого долга группы в таблице нет. Это не «скрыли крах», а просто не публикуют общую картину. По юрлицу «Альфа-М» (это К&amp;Б) наоборот видно: с убытка 2024 вышли на прибыль 26 млрд при выручке 847 млрд. Владельцы сняли большие дивиденды — так делают, когда кэш есть, а не когда спасают сеть. В начале 2026 К&amp;Б впервые чуть сократила число магазинов (минус 4 точки) — это замедление, не развал.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>П.5. Производители: почему PepsiCo и Русагро почти вничью</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>INFOLine сложил выручку десяти крупнейших производителей еды и напитков за 2025 — получилось 3 трлн ₽, рост всего +9,1%. Ритейл (топ-10 сетей) рос быстрее, на 16%. То есть полка увеличивалась сильнее, чем отгрузки заводов: сети отъедают долю за счёт СТМ и дискаунтера, заводам расти труднее.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="96" customHeight="1">
+    <row r="18" ht="64" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Первое и второе место — фотофиниш. PepsiCo Россия 398,8 млрд (+11,1%): напитки, снеки и молочка «Вимм-Билль-Данн». Русагро 396,5 млрд (+16,6%) — почти догнала. Рост Русагро не «масло лучше продалось», а сделка: в периметр полностью вошло «Агро-Белогорье», мясная выручка +71%. Чистая прибыль Русагро при этом упала в 1,6 раза до 19,9 млрд: льготные сельхозкредиты подорожали, рубль окреп — на валютной подушке и экспортной дебиторке получили курсовой минус. Долг вырос. Гендиректор Тимур Липатов это прямо сказал в отчётности (Интерфакс 06.03.2026; презентация Русагро 12М 2025).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="88" customHeight="1">
+          <t>Теперь другая сторона прилавка — кто кладёт еду и напитки на полку, а не кто её продаёт. INFOLine сложил выручку десяти крупнейших производителей за 2025 год: 3 трлн ₽, рост всего на 9,1%. Сети (топ-10) росли быстрее — примерно на 16%. Простыми словами: полка в магазине увеличивалась сильнее, чем отгрузки заводов. Сети отъедают долю своими марками (СТМ) и дискаунтерами, заводам расти труднее.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="120" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Что изменилось в десятке. Раньше наверху стояли глобальные бренды (PepsiCo, Nestlé, Mars). Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка»: Русагро, Мираторг, Черкизово, ГАП Ресурс, Агропромкомплектация. Они сами выращивают, сами режут, сами кладут на полку. Для сетей это значит: переговоры всё чаще с вертикальным холдингом, а не с «просто поставщиком соуса». ЭФКО (3-е место) выручку не нарастила (0%). KDV почти остановилась (+1%). Черкизово: выручка +11,4% до 289 млрд, прибыль 30 млрд, но «очищенная» прибыль даже чуть снизилась (−4,4% до 19,5) — красивая цифра 30 млрд включает переоценку биоактивов. Долг 140 млрд, 2,5× EBITDA, за год почти не вырос.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+          <t>Первое и второе место — почти фотофиниш. PepsiCo Россия продала на 398,8 млрд ₽ (+11,1%): это Pepsi, Lay's и молочка «Вимм-Билль-Данн». Русагро — 396,5 млрд (+16,6%), то есть отстала меньше чем на 3 млрд. Но Русагро догнала не потому, что масло вдруг стали лучше брать. В периметр полностью вошло «Агро-Белогорье», мясная выручка подскочила на 71%. Это рост «купили завод», а не «масло лучше продалось».
+При этом заработать Русагро стала меньше: прибыль упала в 1,6 раза, до 19,9 млрд. Льготные сельхозкредиты подорожали, рубль окреп — на валютной подушке и долгах покупателей из-за рубежа получился курсовой минус. Долг вырос. Гендиректор Тимур Липатов это прямо сказал в отчётности (Интерфакс 06.03.2026; презентация Русагро за 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="112" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Что изменилось в десятке. Раньше наверху стояли глобальные бренды: PepsiCo, Nestlé, Mars. Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка»: Русагро, Мираторг, Черкизово, ГАП Ресурс, Агропромкомплектация. Они сами выращивают, сами режут, сами кладут на полку. Для закупщика сети это значит: торгуешься уже не с «просто поставщиком соуса», а с вертикальным холдингом.
+Не у всех год был про рост. ЭФКО (третье место) выручку не нарастила совсем — ноль. KDV почти остановилась (+1%). Черкизово продала на 11% больше (289 млрд), в отчёте прибыль 30 млрд. Но «очищенная» прибыль — без переоценки свиней и кур на балансе — 19,5 млрд, чуть ниже прошлого года. Красивая цифра 30 млрд включает бумажную переоценку. Долг 140 млрд, примерно 2,5 года прибыли, за год почти не вырос.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>П.6. Молочка и пиво: кто теперь первый на полке</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="112" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Молочка. Несколько лет лидером рейтинга Союзмолоко / Milknews был «Вимм-Билль-Данн» (это кусок PepsiCo: «Домик в деревне», «Чудо» и т.д.). В 2025 первое место впервые взяла «Логика молока» — 167,1 млрд ₽ (+17,9%) против 162,3 млрд у ВБД (+6,7%). Кто это: бывшие заводы Danone («Простоквашино», «Растишка», «Актибио», «Тема»), с 2024 под российским контролем. Почему обогнали: росли быстрее весь год, а в декабре докупили мороженое «Новосибхолод» / «Полярис» — и вырвались. Важно: 162,3 млрд ВБД уже сидят внутри PepsiCo 398,8 на листе производителей. Отдельную строку ВБД смотрите в «Вывесках», не прибавляйте к PepsiCo. Источник: Союзмолоко / Интерфакс 21.07.2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="64" customHeight="1">
+    <row r="23" ht="120" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Пиво. «Напитки вместе» (так теперь называется бывший AB InBev Efes в России) — 164,7 млрд (+16,6%), INFOLine ставит их на границу топ-10/20 еды и напитков, по пиву это №1. «Балтика» (бывший Carlsberg, тоже российский контур): выручка юрлица 145,9 млрд (+8,2%) и прибыль 13,3 млрд — годом раньше компания была убыточной, в 2025 вышла в плюс. Для полки: оба больших пивных контура остались, сменились вывески и собственники, а не исчезли бренды.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n"/>
-    </row>
-    <row r="25" ht="56" customHeight="1">
+          <t>Молочка. Несколько лет в рейтинге Союзмолоко первым был «Вимм-Билль-Данн» — это кусок PepsiCo, «Домик в деревне», «Чудо» и так далее. В 2025 году первое место впервые взяла «Логика молока»: 167,1 млрд ₽ против 162,3 млрд у ВБД. Кто это такие: бывшие заводы Danone — «Простоквашино», «Растишка», «Актибио», «Тема». С 2024 года они под российским контролем.
+Почему обогнали: росли быстрее весь год (+17,9% против +6,7% у ВБД), а в декабре докупили мороженое «Новосибхолод» / «Полярис» — и этого хватило, чтобы вырваться. Важно для таблицы: 162 млрд ВБД уже сидят внутри PepsiCo (398 млрд) на листе производителей. Отдельную строку ВБД нельзя прибавлять к PepsiCo — получится двойной счёт. Источник: Союзмолоко / Интерфакс 21.07.2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Пиво. Бывший AB InBev Efes в России теперь называется «Напитки вместе»: 164,7 млрд ₽ (+16,6%). По пиву это первый. «Балтика» (бывший Carlsberg, тоже уже российский контур) — 145,9 млрд (+8,2%) и прибыль 13,3 млрд. Годом раньше Балтика была убыточной, в 2025 вышла в плюс. Для полки это значит: оба больших пивных контура никуда не делись. Сменились вывески и собственники, а не исчезли бренды в холодильнике.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="88" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Ещё два факта коротко. Хард-дискаунтер: Чижик внутри X5 +67% до 418 млрд, а «Светофор» −3% и минус 315 магазинов. Формат жив, конкретный бренд «Светофор» сжимается (конкуренция + проверки Роспотребнадзора, «Ъ» / Ведомости). Регионалы с твёрдой выручкой &gt;100 млрд: Верный 154, SPAR Миддл Волга 136, Мария-Ра 128, Ермолино ~111, Командор 100 — зона возможных сделок, не зона спокойного автономного роста.</t>
+          <t>Ещё два факта, которые часто путают.
+Хард-дискаунтер как формат не умер. «Чижик» внутри X5 вырос на 67% и дошёл до 418 млрд ₽. А вот сам «Светофор» сжался: выручка −3%, закрыли 315 магазинов. Формат жив, конкретный бренд «Светофор» сжимается — конкуренция с Чижиком плюс проверки Роспотребнадзора.
+Региональные сети с выручкой больше 100 млрд — Верный 154, SPAR Миддл Волга 136, Мария-Ра 128, Ермолино около 111, Командор 100 — это не «маленькие спокойные магазинчики». Это как раз тот размер, на который крупные группы смотрят как на возможные покупки, а не зона, где можно годы расти самим и тебя не тронут.</t>
         </is>
       </c>
     </row>
@@ -6678,24 +6694,24 @@
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="78" customWidth="1" min="3" max="3"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Открытые разборы по топ-10: что читать и зачем</t>
+          <t>Разборы топ-10: что случилось, человеческим языком</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="52" customHeight="1">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Не рейтинг и не таблица цифр. Это статьи и отчёты, которые объясняют, почему у компании сейчас так, а не иначе. Цифра в файле берётся из отчётности; статья — чтобы понять сюжет.</t>
+          <t>Это не рейтинг и не таблица цифр. Ниже — сюжет каждой компании словами: что произошло в 2025 году, почему так, и чем это не является (например, не «магазины опустели»). Цифры в таблицах «Сети» / «Производители» берутся из отчётности; колонка справа — статья, если захотите дочитать. Все сравнения — 2025 к 2024. Годового 2026 ещё нет.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6730,7 +6746,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="56" customHeight="1">
+    <row r="5" ht="132" customHeight="1">
       <c r="A5" s="25" t="n">
         <v>1</v>
       </c>
@@ -6741,7 +6757,7 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Касса +19%, прибыль −14%. Причина не в пустых магазинах, а в процентах по долгу, резерве 4,1 млрд и больших дивидендах/байбеке.</t>
+          <t>Люди в Пятёрочку, Перекрёсток и Чижик ходили как ходили: за год в кассах оказалось 4,64 трлн ₽ — на 19% больше, чем в 2024-м. Казалось бы, отличный год. Но в карман компании легло меньше: чистая прибыль упала на 14%, до 94,8 млрд. Почему так, если магазины не пустые? Три понятные причины. Первая — кредиты стали дороже, и тело долга больше, поэтому банкам ушло больше процентов. Вторая — разово отложили 4,1 млрд «на всякий случай», если кто-то из партнёров не расплатится. Третья — владельцам щедро вернули деньги: дивиденды около 159 млрд и выкуп своих акций около 45 млрд. Это не дыра в магазинах, а раздача кэша акционерам. Коротко: полка живая, меньше стало не покупок, а того, что осталось после банков и дивидендов.</t>
         </is>
       </c>
       <c r="D5" s="28" t="inlineStr">
@@ -6750,7 +6766,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="56" customHeight="1">
+    <row r="6" ht="132" customHeight="1">
       <c r="A6" s="25" t="n">
         <v>2</v>
       </c>
@@ -6761,7 +6777,7 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Касса +15%, но убыток 16,6 млрд. Дорогой долг (ставка 17,1%), покупка «Азбуки вкуса» и «Самбери». «Тандер» — первый убыток за 20 лет. Сеть при этом работает.</t>
+          <t>Та же история на кассе и другая внизу отчёта. Выручка выросла на 15%, до 3,51 трлн ₽ — люди покупали. А прибыли нет: убыток 16,6 млрд. Годом раньше была прибыль около 50 млрд. То есть за один год компания перешла из «заработали» в «ушли в минус», хотя магазины не опустели. Деньги в 2025 году стоили очень дорого: средняя ставка по долгу 17,1%, одних процентов набежало больше 82 млрд. Плюс купили «Азбуку вкуса» и «Самбери». Юрлицо, которое реально крутит магазины, — «Тандер» — впервые за двадцать с лишним лет закончило год в минусе. Это не «покупатели ушли». Это проценты по кредитам съели результат. Около 33 тысяч магазинов при этом работают.</t>
         </is>
       </c>
       <c r="D6" s="28" t="inlineStr">
@@ -6770,7 +6786,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="56" customHeight="1">
+    <row r="7" ht="132" customHeight="1">
       <c r="A7" s="25" t="n">
         <v>3</v>
       </c>
@@ -6781,7 +6797,7 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Чистый долг ×2 до 496 млрд. Половина — банки, половина — облигации на бирже. Компания говорит: заняли заранее, чтобы закрыть погашения 2026-го.</t>
+          <t>У Магнита самый тяжёлый рюкзак из крупных сетей: чистый долг почти удвоился и дошёл до 496 млрд ₽. Весь долг ещё больше — 746 млрд. Примерно половина — кредиты банков, половина — облигации на Московской бирже (их купили фонды, банки, частные инвесторы; поимённый список компания не публикует, так устроен рынок). Сама компания говорит: во втором полугодии нарочно набрала лишних денег, чтобы заранее закрыть погашения 2026 года, а не потому что в кассах кончились деньги. Признаков дефолта нет: магазины работают, отчётность выходит, облигации торгуются. Но это уже не спокойный долг. Если ставка останется высокой, проценты будут и дальше съедать прибыль. За чем следить: сможет ли перекредитоваться дешевле.</t>
         </is>
       </c>
       <c r="D7" s="28" t="inlineStr">
@@ -6790,7 +6806,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="56" customHeight="1">
+    <row r="8" ht="132" customHeight="1">
       <c r="A8" s="25" t="n">
         <v>4</v>
       </c>
@@ -6801,7 +6817,7 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>И выручка, и прибыль выросли. Долг 48,8 млрд упал, 0,6× EBITDA. Весь долг — кредиты банков, не облигации. Рейтинг AA+. К краху не похоже.</t>
+          <t>Полная противоположность Магниту. И выручка выросла, и прибыль выросла. Чистый долг не раздулся, а наоборот упал: было 60,9 млрд, стало 48,8. Это в 23 раза меньше, чем у Магнита. Закрыть такой долг хватило бы меньше чем года обычной прибыли. Перед кем должна: только банкам, облигаций в 2025 ещё не было. На счетах лежит 51 млрд кэша — почти столько же, сколько короткий долг. Три рейтинговых агентства весной 2026 поставили оценки уровня AA+: «высокая надёжность». Развалится ли сеть? По открытым данным — нет. Долг появился как у любой крупной сети: товар на складе, стройка магазинов, покупка «Монетки», «Реми», «Улыбки радуги». Это рабочий инструмент, не признак краха.</t>
         </is>
       </c>
       <c r="D8" s="28" t="inlineStr">
@@ -6810,7 +6826,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="56" customHeight="1">
+    <row r="9" ht="132" customHeight="1">
       <c r="A9" s="25" t="n">
         <v>5</v>
       </c>
@@ -6821,7 +6837,7 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Сама компания: выручка 1,1 трлн, долг/EBITDA 0,6×, кэш 51 млрд. Драйверы — «Монетка», супермаркеты, сделки.</t>
+          <t>То же самое словами самой компании. В годовом отчёте за 2025-й: выручка 1,1 трлн ₽, прибыль 38,2 млрд, на счетах 51 млрд. Рост дали «Монетка», супермаркеты и купленные вывески. Этот отчёт — первоисточник к строке «Лента» в таблице, а не пересказ чужих слухов.</t>
         </is>
       </c>
       <c r="D9" s="28" t="inlineStr">
@@ -6830,7 +6846,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="56" customHeight="1">
+    <row r="10" ht="132" customHeight="1">
       <c r="A10" s="25" t="n">
         <v>6</v>
       </c>
@@ -6841,7 +6857,7 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Холдинг +20% до 1,66 трлн. «Альфа-М» вышла из убытка на 26 млрд прибыли. Владельцы сняли крупные дивиденды — признак кэша, не спасения.</t>
+          <t>«Красное &amp; Белое» плюс «Бристоль» вместе продали на 1,66 трлн ₽ — на 20% больше, чем годом раньше. Сводного отчёта на весь холдинг нет, поэтому чистого долга группы в таблице нет: это не «скрыли крах», а просто не публикуют общую картину. Зато по юрлицу «Альфа-М» (это К&amp;Б) видно: с убытка 2024 года вышли на прибыль 26 млрд. Владельцы сняли большие дивиденды — десятки миллиардов. Так делают, когда кэш есть, а не когда спасают сеть. В начале 2026-го К&amp;Б впервые чуть сократила число магазинов (минус 4 точки). Это замедление, не развал.</t>
         </is>
       </c>
       <c r="D10" s="28" t="inlineStr">
@@ -6850,7 +6866,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="56" customHeight="1">
+    <row r="11" ht="132" customHeight="1">
       <c r="A11" s="25" t="n">
         <v>7</v>
       </c>
@@ -6861,7 +6877,7 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Выручка −3%, закрыли 315 магазинов. Не «формат умер»: Чижик у X5 +67%. У Торгсервиса — конкуренция, качество точек и проверки Роспотребнадзора.</t>
+          <t>Единственный крупный хард-дискаунтер, который сжался. Выручка −3%, закрыли 315 магазинов. Из этого часто делают вывод «формат дешёвых магазинов умер». Это не так. Формат жив: «Чижик» внутри X5 вырос на 67% и дошёл до 418 млрд ₽. У самого «Светофора» своя история: конкуренция с Чижиком, вопросы к качеству части точек и проверки Роспотребнадзора. Коротко: дешёвый магазин у дома никуда не делся, сжался конкретный бренд «Светофор».</t>
         </is>
       </c>
       <c r="D11" s="28" t="inlineStr">
@@ -6870,7 +6886,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="56" customHeight="1">
+    <row r="12" ht="132" customHeight="1">
       <c r="A12" s="25" t="n">
         <v>8</v>
       </c>
@@ -6881,7 +6897,7 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Фотофиниш 399 vs 397 млрд. Русагро догнала за счёт «Агро-Белогорья», но прибыль −1,6×: дорогие льготные кредиты и курс рубля.</t>
+          <t>Два гиганта еды закончили год почти вничью: PepsiCo Россия 399 млрд ₽, Русагро 397. PepsiCo — это напитки, снеки и молочка «Вимм-Билль-Данн». Русагро догнала не потому, что масло вдруг стали лучше брать. В компанию полностью вошло «Агро-Белогорье», мясная выручка подскочила на 71%. Это рост «купили завод», а не «полка лучше продалась». При этом заработать Русагро стала меньше: прибыль упала в 1,6 раза, до 19,9 млрд. Льготные сельхозкредиты подорожали, рубль окреп — на валютной подушке получился минус. Долг вырос. Продаж почти как у PepsiCo, денег в кармане — меньше.</t>
         </is>
       </c>
       <c r="D12" s="28" t="inlineStr">
@@ -6890,7 +6906,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="56" customHeight="1">
+    <row r="13" ht="132" customHeight="1">
       <c r="A13" s="25" t="n">
         <v>9</v>
       </c>
@@ -6901,7 +6917,7 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Выручка +11%, прибыль 30 млрд (очищенная 19,5, чуть ниже). Долг 140 млрд почти не вырос, нагрузка 2,5× с 3,0×.</t>
+          <t>Продали на 11% больше — 289 млрд ₽. В заголовках часто пишут «прибыль 30 млрд», и это звучит как праздник. Но если убрать бумажную переоценку свиней и кур на балансе, «очищенная» прибыль 19,5 млрд — даже чуть ниже, чем годом раньше. Долг 140 млрд, примерно 2,5 года обычной прибыли, за год почти не вырос. Картина спокойная, не рывок и не провал.</t>
         </is>
       </c>
       <c r="D13" s="28" t="inlineStr">
@@ -6910,7 +6926,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="56" customHeight="1">
+    <row r="14" ht="132" customHeight="1">
       <c r="A14" s="25" t="n">
         <v>10</v>
       </c>
@@ -6921,7 +6937,7 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Впервые лидер молочки — не PepsiCo. «Логика молока» (ex-Danone) 167 млрд обошла ВБД 162 млрд: быстрее росла и купила мороженое в декабре.</t>
+          <t>Несколько лет молочную полку по выручке возглавлял «Вимм-Билль-Данн» — это кусок PepsiCo, «Домик в деревне», «Чудо». В 2025-м первое место впервые взяла «Логика молока»: 167 млрд против 162 млрд у ВБД. Кто это: бывшие заводы Danone — «Простоквашино», «Растишка», «Тема». С 2024 года они под российским контролем. Почему обогнали: весь год росли быстрее, а в декабре докупили мороженое «Новосибхолод» / «Полярис» — и этого хватило, чтобы вырваться. Важно: 162 млрд ВБД уже входят в 399 млрд PepsiCo. Складывать их ещё раз нельзя — получится двойной счёт.</t>
         </is>
       </c>
       <c r="D14" s="28" t="inlineStr">
@@ -6930,7 +6946,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="56" customHeight="1">
+    <row r="15" ht="132" customHeight="1">
       <c r="A15" s="25" t="n">
         <v>11</v>
       </c>
@@ -6941,7 +6957,7 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Десять заводов вместе 3 трлн (+9,1%). В десятке уже пять агрохолдингов. ЭФКО без роста, KDV +1%.</t>
+          <t>Десять крупнейших производителей еды и напитков вместе отгрузили на 3 трлн ₽ — рост всего 9%. Сети при этом росли примерно на 16%. Простыми словами: полка в магазине увеличивалась быстрее, чем заводы успевали отгружать. Сети отъедают долю своими марками и дискаунтерами, заводам расти труднее. Раньше наверху стояли глобальные бренды. Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка». Не у всех год был про рост: ЭФКО выручку не нарастила совсем, KDV почти остановилась (+1%).</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">
@@ -6950,7 +6966,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="56" customHeight="1">
+    <row r="16" ht="132" customHeight="1">
       <c r="A16" s="25" t="n">
         <v>12</v>
       </c>
@@ -6961,7 +6977,7 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Первый убыток операционной компании с начала 2000-х. Магнит объясняет капвложениями и ставкой, не падением трафика.</t>
+          <t>«Тандер» — это не отдельная сеть на полке, а юрлицо, которое реально крутит магазины «Магнита». В 2025 году оно впервые с начала 2000-х закончило год с убытком (порядка 22 млрд). Заголовки звучат страшно, смысл тот же, что у всей группы: не «покупатели разбежались», а дорогие кредиты и вложения в развитие. Магнит сам так и объясняет. Магазины при этом работают. Это тот же сюжет, что в строке «Магнит», только на уровне конкретной компании в ЕГРЮЛ.</t>
         </is>
       </c>
       <c r="D16" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Clarify that STM and discounters shift brand margin, not who makes the food
The old wording sounded as if chains produce groceries instead of factories.
Spell out: goods still come from plants; what changes is the name on the pack
and which factory (brand owner vs contract) captures the sale.

Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_sentyabr_2026.xlsx
+++ b/FMCG_RF_sentyabr_2026.xlsx
@@ -1195,10 +1195,10 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="64" customHeight="1">
+    <row r="18" ht="96" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Теперь другая сторона прилавка — кто кладёт еду и напитки на полку, а не кто её продаёт. INFOLine сложил выручку десяти крупнейших производителей за 2025 год: 3 трлн ₽, рост всего на 9,1%. Сети (топ-10) росли быстрее — примерно на 16%. Простыми словами: полка в магазине увеличивалась сильнее, чем отгрузки заводов. Сети отъедают долю своими марками (СТМ) и дискаунтерами, заводам расти труднее.</t>
+          <t>Теперь другая сторона прилавка — кто кладёт еду и напитки на полку, а не кто её продаёт. INFOLine сложил выручку десяти крупнейших производителей за 2025 год: 3 трлн ₽, рост всего на 9,1%. Сети (топ-10) росли быстрее — примерно на 16%. Товар по-прежнему приходит с заводов: сеть сама молоко не доит. Меняется имя на пачке и то, кто забирает наценку. Раньше на полке чаще стоял бренд завода (Pepsi, «Домик в деревне», Lay's) — деньги за бренд шли производителю. Сейчас всё больше пачек с маркой магазина (СТМ: «Красная цена», «Пятёрочка» и т.п.). Их тоже сварил какой-то завод, но часто другой, контрактный, или тот же — только без брендовой цены. В дискаунтере (Чижик) полка короткая: брендам именитых заводов просто меньше места. Поэтому кассы сетей растут быстрее, чем выручка десятки известных производителей.</t>
         </is>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Десять крупнейших производителей еды и напитков вместе отгрузили на 3 трлн ₽ — рост всего 9%. Сети при этом росли примерно на 16%. Простыми словами: полка в магазине увеличивалась быстрее, чем заводы успевали отгружать. Сети отъедают долю своими марками и дискаунтерами, заводам расти труднее. Раньше наверху стояли глобальные бренды. Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка». Не у всех год был про рост: ЭФКО выручку не нарастила совсем, KDV почти остановилась (+1%).</t>
+          <t>Десять крупнейших производителей еды и напитков вместе отгрузили на 3 трлн ₽ — рост всего 9%. Сети при этом росли примерно на 16%. Товар по-прежнему везут с заводов: сеть сама еду не производит (кроме редких своих цехов). Меняется другое: на пачке всё чаще марка магазина, а не Pepsi или «Домик в деревне». Завод есть, но это часто контрактный завод или тот же без брендовой наценки. В дискаунтере короткая полка — брендам меньше места. Поэтому кассы сетей растут быстрее, чем выручка известных заводов из рейтинга. Раньше наверху стояли глобальные бренды. Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка». Не у всех год был про рост: ЭФКО выручку не нарастила совсем, KDV почти остановилась (+1%).</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">

</xml_diff>

<commit_message>
Shorten the private-label explanation to a few plain sentences
Co-authored-by: Alena931 <Alena931@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/FMCG_RF_sentyabr_2026.xlsx
+++ b/FMCG_RF_sentyabr_2026.xlsx
@@ -1195,10 +1195,10 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="96" customHeight="1">
+    <row r="18" ht="80" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>Теперь другая сторона прилавка — кто кладёт еду и напитки на полку, а не кто её продаёт. INFOLine сложил выручку десяти крупнейших производителей за 2025 год: 3 трлн ₽, рост всего на 9,1%. Сети (топ-10) росли быстрее — примерно на 16%. Товар по-прежнему приходит с заводов: сеть сама молоко не доит. Меняется имя на пачке и то, кто забирает наценку. Раньше на полке чаще стоял бренд завода (Pepsi, «Домик в деревне», Lay's) — деньги за бренд шли производителю. Сейчас всё больше пачек с маркой магазина (СТМ: «Красная цена», «Пятёрочка» и т.п.). Их тоже сварил какой-то завод, но часто другой, контрактный, или тот же — только без брендовой цены. В дискаунтере (Чижик) полка короткая: брендам именитых заводов просто меньше места. Поэтому кассы сетей растут быстрее, чем выручка десятки известных производителей.</t>
+          <t>Теперь другая сторона прилавка — кто кладёт еду и напитки на полку, а не кто её продаёт. INFOLine сложил выручку десяти крупнейших производителей за 2025 год: 3 трлн ₽, рост всего на 9,1%. Сети (топ-10) росли быстрее — примерно на 16%. Еду по-прежнему варит завод, сеть сама её не делает. Меняется имя на пачке: вместо Lay's или «Домик в деревне» всё чаще марка магазина («Пятёрочка», «Красная цена»). Деньги за бренд тогда идут сети, а не известному заводу. В дешёвом магазине вроде Чижика к тому же короткая полка — брендам просто меньше места. Поэтому кассы сетей растут быстрее, чем выручка больших брендов.</t>
         </is>
       </c>
     </row>
@@ -6957,7 +6957,7 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Десять крупнейших производителей еды и напитков вместе отгрузили на 3 трлн ₽ — рост всего 9%. Сети при этом росли примерно на 16%. Товар по-прежнему везут с заводов: сеть сама еду не производит (кроме редких своих цехов). Меняется другое: на пачке всё чаще марка магазина, а не Pepsi или «Домик в деревне». Завод есть, но это часто контрактный завод или тот же без брендовой наценки. В дискаунтере короткая полка — брендам меньше места. Поэтому кассы сетей растут быстрее, чем выручка известных заводов из рейтинга. Раньше наверху стояли глобальные бренды. Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка». Не у всех год был про рост: ЭФКО выручку не нарастила совсем, KDV почти остановилась (+1%).</t>
+          <t>Десять крупнейших производителей еды и напитков вместе отгрузили на 3 трлн ₽ — рост всего 9%. Сети при этом росли примерно на 16%. Еду по-прежнему варит завод, сеть сама её не делает. Меняется имя на пачке: вместо Lay's или «Домик в деревне» всё чаще марка магазина. Деньги за бренд тогда идут сети, а не известному заводу. В дешёвом магазине вроде Чижика брендам ещё и меньше места на полке. Поэтому кассы сетей растут быстрее, чем выручка больших брендов. Раньше наверху стояли глобальные марки. Сейчас пять из десяти — российские агрохолдинги «от поля до прилавка». Не у всех год был про рост: ЭФКО выручку не нарастила совсем, KDV почти остановилась (+1%).</t>
         </is>
       </c>
       <c r="D15" s="28" t="inlineStr">

</xml_diff>